<commit_message>
reimplemented PlatformsList as Datasets, which reads an excel file
</commit_message>
<xml_diff>
--- a/datasets_info.xlsx
+++ b/datasets_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\punge\DownSyndromeCuration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D89387AB-6B49-49F5-AC16-CD4AD40B4EBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5DBAFD7-6C07-4E25-83D8-7B8DB5316A57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{921AEB32-BBE2-40F1-B29F-64DEE11BC5B8}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" xr2:uid="{921AEB32-BBE2-40F1-B29F-64DEE11BC5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="41">
   <si>
     <t>Name</t>
   </si>
@@ -120,9 +120,6 @@
   </si>
   <si>
     <t>RNA</t>
-  </si>
-  <si>
-    <t>NA</t>
   </si>
   <si>
     <t>mouse</t>
@@ -554,7 +551,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -565,13 +562,10 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -582,9 +576,6 @@
         <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" t="s">
         <v>28</v>
       </c>
     </row>
@@ -596,9 +587,6 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" t="s">
         <v>28</v>
       </c>
     </row>
@@ -610,13 +598,10 @@
         <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" t="s">
         <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -627,10 +612,7 @@
         <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -641,9 +623,6 @@
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -655,9 +634,6 @@
         <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" t="s">
         <v>28</v>
       </c>
     </row>
@@ -666,13 +642,13 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" t="s">
         <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -680,13 +656,13 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" t="s">
         <v>31</v>
-      </c>
-      <c r="C10" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -694,13 +670,13 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" t="s">
         <v>31</v>
-      </c>
-      <c r="C11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -708,13 +684,13 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -722,13 +698,13 @@
         <v>19</v>
       </c>
       <c r="B13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" t="s">
         <v>31</v>
-      </c>
-      <c r="C13" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -736,13 +712,13 @@
         <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -750,16 +726,16 @@
         <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -767,13 +743,13 @@
         <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -781,13 +757,13 @@
         <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -795,13 +771,13 @@
         <v>24</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -809,13 +785,13 @@
         <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -823,13 +799,13 @@
         <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C20" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -837,13 +813,13 @@
         <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -851,13 +827,13 @@
         <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -865,13 +841,13 @@
         <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -879,13 +855,13 @@
         <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
saved changes to GSEs
</commit_message>
<xml_diff>
--- a/datasets_info.xlsx
+++ b/datasets_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\punge\DownSyndromeCuration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DDEBF41-E81F-4B69-9D6B-B6BD534285CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF8EC47-C26E-4BF4-BCF9-A857CD86D123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6984" yWindow="3336" windowWidth="9300" windowHeight="7848" xr2:uid="{921AEB32-BBE2-40F1-B29F-64DEE11BC5B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{921AEB32-BBE2-40F1-B29F-64DEE11BC5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="87">
   <si>
     <t>Name</t>
   </si>
@@ -161,14 +161,149 @@
     <t>Needs both platforms c("GPL570", "GPL96")</t>
   </si>
   <si>
-    <t>missing ones</t>
+    <t>GSE114559</t>
+  </si>
+  <si>
+    <t>GSE121065</t>
+  </si>
+  <si>
+    <t>GSE121066</t>
+  </si>
+  <si>
+    <t>GSE124252</t>
+  </si>
+  <si>
+    <t>GSE124513</t>
+  </si>
+  <si>
+    <t>GSE125837</t>
+  </si>
+  <si>
+    <t>GSE126910</t>
+  </si>
+  <si>
+    <t>GSE128614</t>
+  </si>
+  <si>
+    <t>GSE128621</t>
+  </si>
+  <si>
+    <t>GSE131249</t>
+  </si>
+  <si>
+    <t>GSE137939</t>
+  </si>
+  <si>
+    <t>GSE138371</t>
+  </si>
+  <si>
+    <t>GSE138468</t>
+  </si>
+  <si>
+    <t>GSE139285</t>
+  </si>
+  <si>
+    <t>GSE144857</t>
+  </si>
+  <si>
+    <t>GSE151255</t>
+  </si>
+  <si>
+    <t>GSE151282</t>
+  </si>
+  <si>
+    <t>GSE154418</t>
+  </si>
+  <si>
+    <t>GSE160637</t>
+  </si>
+  <si>
+    <t>GSE160690</t>
+  </si>
+  <si>
+    <t>GSE166849</t>
+  </si>
+  <si>
+    <t>GSE167021</t>
+  </si>
+  <si>
+    <t>GSE175539</t>
+  </si>
+  <si>
+    <t>GSE183701</t>
+  </si>
+  <si>
+    <t>GSE185192</t>
+  </si>
+  <si>
+    <t>GSE188568</t>
+  </si>
+  <si>
+    <t>GSE189225</t>
+  </si>
+  <si>
+    <t>GSE190305</t>
+  </si>
+  <si>
+    <t>GSE201093</t>
+  </si>
+  <si>
+    <t>GSE201290</t>
+  </si>
+  <si>
+    <t>GSE203257</t>
+  </si>
+  <si>
+    <t>GSE208575</t>
+  </si>
+  <si>
+    <t>GSE213500</t>
+  </si>
+  <si>
+    <t>GSE213502</t>
+  </si>
+  <si>
+    <t>GSE222365</t>
+  </si>
+  <si>
+    <t>GSE229563</t>
+  </si>
+  <si>
+    <t>GSE42142</t>
+  </si>
+  <si>
+    <t>GSE52249</t>
+  </si>
+  <si>
+    <t>GSE55504</t>
+  </si>
+  <si>
+    <t>GSE64840</t>
+  </si>
+  <si>
+    <t>GSE79842</t>
+  </si>
+  <si>
+    <t>GSE84526</t>
+  </si>
+  <si>
+    <t>GSE84531</t>
+  </si>
+  <si>
+    <t>GSE95551</t>
+  </si>
+  <si>
+    <t>GSE95552</t>
+  </si>
+  <si>
+    <t>Two SRR/GSM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -176,16 +311,34 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -193,12 +346,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -533,7 +707,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54585A14-21B9-4C53-99B4-04DAE4E266F3}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" customWidth="1"/>
@@ -629,7 +803,7 @@
         <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>41</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -856,7 +1030,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -868,6 +1042,501 @@
       </c>
       <c r="D24" t="s">
         <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B31" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B32" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B33" t="s">
+        <v>27</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B35" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B36" t="s">
+        <v>27</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B37" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B38" t="s">
+        <v>27</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B39" t="s">
+        <v>27</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B40" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B41" t="s">
+        <v>27</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B42" t="s">
+        <v>27</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B43" t="s">
+        <v>27</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B44" t="s">
+        <v>27</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B45" t="s">
+        <v>27</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B46" t="s">
+        <v>27</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B47" t="s">
+        <v>27</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B48" t="s">
+        <v>27</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B49" t="s">
+        <v>27</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B50" t="s">
+        <v>27</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B51" t="s">
+        <v>27</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B52" t="s">
+        <v>27</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B53" t="s">
+        <v>27</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B54" t="s">
+        <v>27</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B55" t="s">
+        <v>27</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B56" t="s">
+        <v>27</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B57" t="s">
+        <v>27</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A58" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B58" t="s">
+        <v>27</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A59" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B60" t="s">
+        <v>27</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B61" t="s">
+        <v>27</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B62" t="s">
+        <v>27</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A63" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B63" t="s">
+        <v>27</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A64" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B64" t="s">
+        <v>27</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A65" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B65" t="s">
+        <v>27</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A66" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B66" t="s">
+        <v>27</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A67" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B67" t="s">
+        <v>27</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A68" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B68" t="s">
+        <v>27</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B69" t="s">
+        <v>27</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
moved problem one to the end for now
</commit_message>
<xml_diff>
--- a/datasets_info.xlsx
+++ b/datasets_info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\punge\DownSyndromeCuration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF8EC47-C26E-4BF4-BCF9-A857CD86D123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A35116B-65FE-4180-804A-786A134C616D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{921AEB32-BBE2-40F1-B29F-64DEE11BC5B8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="88">
   <si>
     <t>Name</t>
   </si>
@@ -297,6 +297,9 @@
   </si>
   <si>
     <t>Two SRR/GSM</t>
+  </si>
+  <si>
+    <t>SRR's not found</t>
   </si>
 </sst>
 </file>
@@ -1354,29 +1357,29 @@
     </row>
     <row r="53" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B53" t="s">
         <v>27</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B54" t="s">
         <v>27</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B55" t="s">
         <v>27</v>
@@ -1387,18 +1390,18 @@
     </row>
     <row r="56" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B56" t="s">
         <v>27</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B57" t="s">
         <v>27</v>
@@ -1409,40 +1412,40 @@
     </row>
     <row r="58" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B58" t="s">
         <v>27</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B59" t="s">
         <v>27</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B60" t="s">
         <v>27</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B61" t="s">
         <v>27</v>
@@ -1453,7 +1456,7 @@
     </row>
     <row r="62" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B62" t="s">
         <v>27</v>
@@ -1464,79 +1467,82 @@
     </row>
     <row r="63" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B63" t="s">
         <v>27</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B64" t="s">
         <v>27</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B65" t="s">
         <v>27</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B66" t="s">
         <v>27</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B67" t="s">
         <v>27</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B68" t="s">
         <v>27</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="B69" t="s">
         <v>27</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>29</v>
+      </c>
+      <c r="E69" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
removed problem GSE for now
</commit_message>
<xml_diff>
--- a/datasets_info.xlsx
+++ b/datasets_info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\punge\DownSyndromeCuration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A35116B-65FE-4180-804A-786A134C616D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4746FFCA-6FF4-49D0-BC68-D29C3A7D1F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{921AEB32-BBE2-40F1-B29F-64DEE11BC5B8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="86">
   <si>
     <t>Name</t>
   </si>
@@ -245,9 +245,6 @@
     <t>GSE190305</t>
   </si>
   <si>
-    <t>GSE201093</t>
-  </si>
-  <si>
     <t>GSE201290</t>
   </si>
   <si>
@@ -297,9 +294,6 @@
   </si>
   <si>
     <t>Two SRR/GSM</t>
-  </si>
-  <si>
-    <t>SRR's not found</t>
   </si>
 </sst>
 </file>
@@ -806,7 +800,7 @@
         <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -1357,7 +1351,7 @@
     </row>
     <row r="53" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B53" t="s">
         <v>27</v>
@@ -1368,7 +1362,7 @@
     </row>
     <row r="54" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B54" t="s">
         <v>27</v>
@@ -1379,7 +1373,7 @@
     </row>
     <row r="55" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B55" t="s">
         <v>27</v>
@@ -1390,7 +1384,7 @@
     </row>
     <row r="56" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B56" t="s">
         <v>27</v>
@@ -1401,7 +1395,7 @@
     </row>
     <row r="57" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B57" t="s">
         <v>27</v>
@@ -1412,7 +1406,7 @@
     </row>
     <row r="58" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B58" t="s">
         <v>27</v>
@@ -1423,7 +1417,7 @@
     </row>
     <row r="59" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B59" t="s">
         <v>27</v>
@@ -1434,7 +1428,7 @@
     </row>
     <row r="60" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B60" t="s">
         <v>27</v>
@@ -1445,7 +1439,7 @@
     </row>
     <row r="61" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B61" t="s">
         <v>27</v>
@@ -1456,7 +1450,7 @@
     </row>
     <row r="62" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B62" t="s">
         <v>27</v>
@@ -1467,7 +1461,7 @@
     </row>
     <row r="63" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B63" t="s">
         <v>27</v>
@@ -1478,52 +1472,52 @@
     </row>
     <row r="64" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B64" t="s">
+        <v>27</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A65" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B64" t="s">
-        <v>27</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="2" t="s">
+      <c r="B65" t="s">
+        <v>27</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A66" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B65" t="s">
-        <v>27</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="2" t="s">
+      <c r="B66" t="s">
+        <v>27</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A67" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B66" t="s">
-        <v>27</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="2" t="s">
+      <c r="B67" t="s">
+        <v>27</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A68" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B67" t="s">
-        <v>27</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="B68" t="s">
         <v>27</v>
       </c>
@@ -1531,19 +1525,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B69" t="s">
-        <v>27</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E69" t="s">
-        <v>87</v>
-      </c>
+    <row r="69" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="2"/>
+      <c r="C69" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Uncommenting file download section, resetting to not be detective mode
</commit_message>
<xml_diff>
--- a/datasets_info.xlsx
+++ b/datasets_info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\punge\DownSyndromeCuration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1340139A-0D08-4FA4-9EBE-A5A42A70D31A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC674D8-B12C-4B5E-ACEE-9452FDB361AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6984" yWindow="3336" windowWidth="9300" windowHeight="7848" xr2:uid="{921AEB32-BBE2-40F1-B29F-64DEE11BC5B8}"/>
+    <workbookView xWindow="12120" yWindow="1068" windowWidth="9348" windowHeight="10008" xr2:uid="{921AEB32-BBE2-40F1-B29F-64DEE11BC5B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>